<commit_message>
Remove template cover instructions
</commit_message>
<xml_diff>
--- a/project/template.xlsx
+++ b/project/template.xlsx
@@ -518,209 +518,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>GA4テンプレートの使い方</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>対象はWebの /g/collect 通信。基本項目、標準イベント項目、商品データを定義しています。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>送信項目はイベント・同意状態・実装により異なります。すべての行が送信必須という意味ではありません。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>案件別template.xlsxのGA4シート末尾に行を追加し、A～E列を既存行と同じ形式で記入してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>A列には実際の送信キーを記入します。ep.は文字列イベント項目、epn.は数値イベント項目です。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>ユーザープロパティはup.が文字列、upn.が数値です。GA4画面の表示名ではなく送信キーを指定してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>サイト独自のカスタム項目は初期定義に含めていません。標準項目でもep.で送られるものがあります。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>pr1～pr200は商品ごとの送信文字列を比較します。商品ID・価格などの個別展開は行いません。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>数値項目のepn.とep.は別行です。実際に送信された型の行に値が入ります。不要な行は削除できます。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>内部パラメータは変更される場合があります。未定義キーは案件ごとに追加してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>標準イベント: https://developers.google.com/analytics/devguides/collection/ga4/reference/events</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>拡張計測: https://support.google.com/analytics/answer/9216061</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="48" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Adobe Analyticsテンプレートの使い方</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="48" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>A列はAppMeasurementのクエリキー、B列はxdm内のパス、C列はdataから始まるパスです。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>直接対応する値がない列は空欄です。未送信は欠落とは限りません。ヘッダー・URLパス内の情報は別途確認してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>リンク種別・エラーページ・商品情報は方式間で形式が異なります。値の正規化やAdobe側の集計は再現しません。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>prop1～75、eVar1～250、list1～3は設定用の枠です。各サイトの設計に合わせて項目名・説明を記入してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="48" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>独自XDMを使用する場合はB列を実際のパスに変更してください。初期値はAdobe公式のAnalytics用XDMです。</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="48" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>XDMのカスタムイベントは案件ごとに行を追加します。例: _experience.analytics.event1to100.event1.value</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="48" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>events一覧、XDM eventType、XDMコマース指標は別行で確認します。商品文字列とXDM商品配列も別行です。</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="48" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>AppMeasurementのコンテキストデータは送信形式が階層化されます。任意のキーを追加する前に保存データを確認してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="48" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>DataとXDMが両方ある場合はDataを優先します。Dataの標準名と短縮名の同時指定は避けてください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="48" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Adobe送信キー: https://experienceleague.adobe.com/en/docs/analytics/implementation/validate/query-parameters</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="48" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Adobe XDM対応: https://experienceleague.adobe.com/en/docs/analytics/implementation/aep-edge/xdm-var-mapping</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="48" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Adobe Data対応: https://experienceleague.adobe.com/en/docs/analytics/implementation/aep-edge/data-var-mapping</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="B14:J14"/>
-    <mergeCell ref="B17:J17"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B13:J13"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="B10:J10"/>
-    <mergeCell ref="B28:J28"/>
-    <mergeCell ref="B9:J9"/>
-    <mergeCell ref="B24:J24"/>
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="B32:J32"/>
-    <mergeCell ref="B26:J26"/>
-    <mergeCell ref="B16:J16"/>
-    <mergeCell ref="B25:J25"/>
-    <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B18:J18"/>
-    <mergeCell ref="B27:J27"/>
-    <mergeCell ref="B12:J12"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -744,7 +542,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Adobe公式のWeb計測項目。各方式の送信値を比較します。空欄の対応・案件別設定は表紙を参照。</t>
+          <t>Adobe公式のWeb計測項目。各方式の送信値を比較します。</t>
         </is>
       </c>
     </row>
@@ -10978,7 +10776,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>汎用Web GA4。サイト別項目の追加方法は表紙を参照。未送信項目は空欄。</t>
+          <t>汎用Web GA4。未送信項目は空欄。</t>
         </is>
       </c>
     </row>

</xml_diff>